<commit_message>
Fix v9 formula nesting: store KPI values in ДАННЫЕ sheet
Previous version inlined value+prev formulas into trend cells,
causing deep nesting that Excel rejected (1000+ char formulas).

Now each KPI's curr/prev formulas live in a single ДАННЫЕ cell each.
Dashboard value cells become =ДАННЫЕ!$B$N and trend cells become
=IF(ДАННЫЕ!$B$N>ДАННЫЕ!$C$N,"▲","▼"). Max formula length dropped
from 1038 to 165 chars on the dashboard.

Report sheet now references the same registry by KPI label.

https://claude.ai/code/session_01G17TBGcqnyf8bKEVQfJRW9
</commit_message>
<xml_diff>
--- a/WAY_MARKET_v9.xlsx
+++ b/WAY_MARKET_v9.xlsx
@@ -417,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -604,6 +604,7 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2321,7 +2322,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="96">
+      <c r="A2" s="97">
         <f>НАСТРОЙКИ!E5&amp;" | "&amp;TEXT(TODAY(),"MMMM YYYY")</f>
         <v/>
       </c>
@@ -2350,7 +2351,7 @@
         </is>
       </c>
       <c r="F5" s="25">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <f>ДАННЫЕ!$B$100</f>
         <v/>
       </c>
     </row>
@@ -2361,7 +2362,7 @@
         </is>
       </c>
       <c r="F6" s="26">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <f>ДАННЫЕ!$B$113</f>
         <v/>
       </c>
     </row>
@@ -2372,7 +2373,7 @@
         </is>
       </c>
       <c r="F7" s="25">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+        <f>ДАННЫЕ!$B$114</f>
         <v/>
       </c>
     </row>
@@ -2383,7 +2384,7 @@
         </is>
       </c>
       <c r="F8" s="25">
-        <f>IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <f>ДАННЫЕ!$B$115</f>
         <v/>
       </c>
     </row>
@@ -2394,7 +2395,7 @@
         </is>
       </c>
       <c r="F9" s="25">
-        <f>IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <f>ДАННЫЕ!$B$116</f>
         <v/>
       </c>
     </row>
@@ -2412,7 +2413,7 @@
         </is>
       </c>
       <c r="F12" s="26">
-        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <f>ДАННЫЕ!$B$108</f>
         <v/>
       </c>
     </row>
@@ -2423,7 +2424,7 @@
         </is>
       </c>
       <c r="F13" s="26">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <f>ДАННЫЕ!$B$109</f>
         <v/>
       </c>
     </row>
@@ -2434,7 +2435,7 @@
         </is>
       </c>
       <c r="F14" s="26">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Оплата долга"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <f>ДАННЫЕ!$B$110</f>
         <v/>
       </c>
     </row>
@@ -2445,7 +2446,7 @@
         </is>
       </c>
       <c r="F15" s="26">
-        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)</f>
+        <f>ДАННЫЕ!$B$120</f>
         <v/>
       </c>
     </row>
@@ -2512,7 +2513,7 @@
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="97" t="inlineStr">
+      <c r="A24" s="98" t="inlineStr">
         <is>
           <t>Для экспорта в PDF нажмите  [ЭКСПОРТ PDF]  (макрос VBA)</t>
         </is>
@@ -2587,7 +2588,7 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="98" t="inlineStr">
+      <c r="A2" s="99" t="inlineStr">
         <is>
           <t>Заполните разделы ниже один раз. Все листы подстроятся автоматически.</t>
         </is>
@@ -2606,7 +2607,7 @@
           <t>Название магазина</t>
         </is>
       </c>
-      <c r="E5" s="99" t="inlineStr">
+      <c r="E5" s="100" t="inlineStr">
         <is>
           <t>WAY MARKET №2</t>
         </is>
@@ -2618,7 +2619,7 @@
           <t>Дата начала учёта</t>
         </is>
       </c>
-      <c r="E6" s="100" t="inlineStr">
+      <c r="E6" s="101" t="inlineStr">
         <is>
           <t>01.01.2026</t>
         </is>
@@ -2630,7 +2631,7 @@
           <t>Доля в фонд рентабельности (%)</t>
         </is>
       </c>
-      <c r="E7" s="99" t="inlineStr">
+      <c r="E7" s="100" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -2642,7 +2643,7 @@
           <t>Лимит на закуп (%)</t>
         </is>
       </c>
-      <c r="E8" s="99" t="inlineStr">
+      <c r="E8" s="100" t="inlineStr">
         <is>
           <t>75</t>
         </is>
@@ -2654,7 +2655,7 @@
           <t>Начальный долг поставщикам (₽)</t>
         </is>
       </c>
-      <c r="E9" s="101" t="n">
+      <c r="E9" s="102" t="n">
         <v>500000</v>
       </c>
     </row>
@@ -2664,7 +2665,7 @@
           <t>Округление сумм</t>
         </is>
       </c>
-      <c r="E10" s="99" t="inlineStr">
+      <c r="E10" s="100" t="inlineStr">
         <is>
           <t>До рубля</t>
         </is>
@@ -2676,7 +2677,7 @@
           <t>Период сравнения</t>
         </is>
       </c>
-      <c r="E11" s="99" t="inlineStr">
+      <c r="E11" s="100" t="inlineStr">
         <is>
           <t>Прошлый месяц</t>
         </is>
@@ -2695,7 +2696,7 @@
           <t>Количество смен</t>
         </is>
       </c>
-      <c r="E14" s="102" t="n">
+      <c r="E14" s="103" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2705,7 +2706,7 @@
           <t>Смена ДЕНЬ</t>
         </is>
       </c>
-      <c r="E15" s="103" t="inlineStr">
+      <c r="E15" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2717,7 +2718,7 @@
           <t>Смена ВЕЧЕР</t>
         </is>
       </c>
-      <c r="E16" s="103" t="inlineStr">
+      <c r="E16" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2729,7 +2730,7 @@
           <t>Смена НОЧЬ</t>
         </is>
       </c>
-      <c r="E17" s="103" t="inlineStr">
+      <c r="E17" s="104" t="inlineStr">
         <is>
           <t>Выкл</t>
         </is>
@@ -2748,7 +2749,7 @@
           <t>Эквайринг</t>
         </is>
       </c>
-      <c r="E20" s="103" t="inlineStr">
+      <c r="E20" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2760,7 +2761,7 @@
           <t>Перевод</t>
         </is>
       </c>
-      <c r="E21" s="103" t="inlineStr">
+      <c r="E21" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2772,7 +2773,7 @@
           <t>Онлайн торговля</t>
         </is>
       </c>
-      <c r="E22" s="103" t="inlineStr">
+      <c r="E22" s="104" t="inlineStr">
         <is>
           <t>Выкл</t>
         </is>
@@ -2784,7 +2785,7 @@
           <t>Иман (хозяин)</t>
         </is>
       </c>
-      <c r="E23" s="103" t="inlineStr">
+      <c r="E23" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2796,7 +2797,7 @@
           <t>Выплата с кассы</t>
         </is>
       </c>
-      <c r="E24" s="103" t="inlineStr">
+      <c r="E24" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2815,7 +2816,7 @@
           <t>Сверка по наличке</t>
         </is>
       </c>
-      <c r="E27" s="103" t="inlineStr">
+      <c r="E27" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2827,7 +2828,7 @@
           <t>Сверка по эквайрингу</t>
         </is>
       </c>
-      <c r="E28" s="103" t="inlineStr">
+      <c r="E28" s="104" t="inlineStr">
         <is>
           <t>Выкл</t>
         </is>
@@ -2839,7 +2840,7 @@
           <t>Сверка по переводу</t>
         </is>
       </c>
-      <c r="E29" s="103" t="inlineStr">
+      <c r="E29" s="104" t="inlineStr">
         <is>
           <t>Выкл</t>
         </is>
@@ -2858,7 +2859,7 @@
           <t>Списание товара</t>
         </is>
       </c>
-      <c r="E32" s="103" t="inlineStr">
+      <c r="E32" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2870,7 +2871,7 @@
           <t>Возврат поставщику</t>
         </is>
       </c>
-      <c r="E33" s="103" t="inlineStr">
+      <c r="E33" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2882,7 +2883,7 @@
           <t>Касса утром/вечером (остатки)</t>
         </is>
       </c>
-      <c r="E34" s="103" t="inlineStr">
+      <c r="E34" s="104" t="inlineStr">
         <is>
           <t>Вкл</t>
         </is>
@@ -2901,7 +2902,7 @@
           <t>Расхождение кассы больше (₽)</t>
         </is>
       </c>
-      <c r="E37" s="104" t="n">
+      <c r="E37" s="105" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -2911,7 +2912,7 @@
           <t>Общий долг больше (₽)</t>
         </is>
       </c>
-      <c r="E38" s="104" t="n">
+      <c r="E38" s="105" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -2921,7 +2922,7 @@
           <t>Просрочка больше (дней)</t>
         </is>
       </c>
-      <c r="E39" s="105" t="n">
+      <c r="E39" s="106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2933,29 +2934,29 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="106" t="inlineStr">
+      <c r="A43" s="107" t="inlineStr">
         <is>
           <t>КАССИРЫ</t>
         </is>
       </c>
-      <c r="C43" s="107" t="inlineStr">
+      <c r="C43" s="108" t="inlineStr">
         <is>
           <t>КАТЕГОРИИ</t>
         </is>
       </c>
-      <c r="E43" s="108" t="inlineStr">
+      <c r="E43" s="109" t="inlineStr">
         <is>
           <t>СПОСОБЫ ОПЛАТЫ</t>
         </is>
       </c>
-      <c r="G43" s="109" t="inlineStr">
+      <c r="G43" s="110" t="inlineStr">
         <is>
           <t>ТИПЫ ОПЕРАЦИЙ</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="110" t="inlineStr">
+      <c r="A44" s="111" t="inlineStr">
         <is>
           <t>Иванов А.</t>
         </is>
@@ -2965,12 +2966,12 @@
           <t>Закуп товара</t>
         </is>
       </c>
-      <c r="E44" s="111" t="inlineStr">
+      <c r="E44" s="112" t="inlineStr">
         <is>
           <t>Наличка</t>
         </is>
       </c>
-      <c r="G44" s="112" t="inlineStr">
+      <c r="G44" s="113" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
@@ -2999,7 +3000,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="110" t="inlineStr">
+      <c r="A46" s="111" t="inlineStr">
         <is>
           <t>Сидоров С.</t>
         </is>
@@ -3009,12 +3010,12 @@
           <t>Расходный материал</t>
         </is>
       </c>
-      <c r="E46" s="111" t="inlineStr">
+      <c r="E46" s="112" t="inlineStr">
         <is>
           <t>Перевод</t>
         </is>
       </c>
-      <c r="G46" s="112" t="inlineStr">
+      <c r="G46" s="113" t="inlineStr">
         <is>
           <t>Долг</t>
         </is>
@@ -3043,25 +3044,25 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="113" t="n"/>
+      <c r="A48" s="114" t="n"/>
       <c r="C48" s="44" t="inlineStr">
         <is>
           <t>Аренда</t>
         </is>
       </c>
-      <c r="E48" s="111" t="inlineStr">
+      <c r="E48" s="112" t="inlineStr">
         <is>
           <t>Иман</t>
         </is>
       </c>
-      <c r="G48" s="112" t="inlineStr">
+      <c r="G48" s="113" t="inlineStr">
         <is>
           <t>Расхождение</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="114" t="n"/>
+      <c r="A49" s="115" t="n"/>
       <c r="C49" s="35" t="inlineStr">
         <is>
           <t>Коммунальные</t>
@@ -3079,27 +3080,27 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="113" t="n"/>
+      <c r="A50" s="114" t="n"/>
       <c r="C50" s="44" t="inlineStr">
         <is>
           <t>Налог</t>
         </is>
       </c>
-      <c r="E50" s="115" t="n"/>
-      <c r="G50" s="112" t="inlineStr">
+      <c r="E50" s="116" t="n"/>
+      <c r="G50" s="113" t="inlineStr">
         <is>
           <t>Списание</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="114" t="n"/>
+      <c r="A51" s="115" t="n"/>
       <c r="C51" s="35" t="inlineStr">
         <is>
           <t>Прочие расходы</t>
         </is>
       </c>
-      <c r="E51" s="114" t="n"/>
+      <c r="E51" s="115" t="n"/>
       <c r="G51" s="4" t="inlineStr">
         <is>
           <t>Возврат</t>
@@ -3107,559 +3108,559 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="113" t="n"/>
+      <c r="A52" s="114" t="n"/>
       <c r="C52" s="44" t="inlineStr">
         <is>
           <t>Списание</t>
         </is>
       </c>
-      <c r="E52" s="115" t="n"/>
-      <c r="G52" s="112" t="inlineStr">
+      <c r="E52" s="116" t="n"/>
+      <c r="G52" s="113" t="inlineStr">
         <is>
           <t>Касса</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="114" t="n"/>
+      <c r="A53" s="115" t="n"/>
       <c r="C53" s="35" t="inlineStr">
         <is>
           <t>Возврат</t>
         </is>
       </c>
-      <c r="E53" s="114" t="n"/>
+      <c r="E53" s="115" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="113" t="n"/>
+      <c r="A54" s="114" t="n"/>
       <c r="C54" s="44" t="inlineStr">
         <is>
           <t>Маркетинг</t>
         </is>
       </c>
-      <c r="E54" s="115" t="n"/>
+      <c r="E54" s="116" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="114" t="n"/>
+      <c r="A55" s="115" t="n"/>
       <c r="C55" s="35" t="inlineStr">
         <is>
           <t>Охрана</t>
         </is>
       </c>
-      <c r="E55" s="114" t="n"/>
+      <c r="E55" s="115" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="113" t="n"/>
-      <c r="C56" s="116" t="n"/>
-      <c r="E56" s="115" t="n"/>
+      <c r="A56" s="114" t="n"/>
+      <c r="C56" s="117" t="n"/>
+      <c r="E56" s="116" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="114" t="n"/>
-      <c r="C57" s="114" t="n"/>
-      <c r="E57" s="114" t="n"/>
+      <c r="A57" s="115" t="n"/>
+      <c r="C57" s="115" t="n"/>
+      <c r="E57" s="115" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="113" t="n"/>
-      <c r="C58" s="116" t="n"/>
-      <c r="E58" s="115" t="n"/>
+      <c r="A58" s="114" t="n"/>
+      <c r="C58" s="117" t="n"/>
+      <c r="E58" s="116" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="114" t="n"/>
-      <c r="C59" s="114" t="n"/>
-      <c r="E59" s="114" t="n"/>
+      <c r="A59" s="115" t="n"/>
+      <c r="C59" s="115" t="n"/>
+      <c r="E59" s="115" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="113" t="n"/>
-      <c r="C60" s="116" t="n"/>
-      <c r="E60" s="115" t="n"/>
+      <c r="A60" s="114" t="n"/>
+      <c r="C60" s="117" t="n"/>
+      <c r="E60" s="116" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="114" t="n"/>
-      <c r="C61" s="114" t="n"/>
-      <c r="E61" s="114" t="n"/>
+      <c r="A61" s="115" t="n"/>
+      <c r="C61" s="115" t="n"/>
+      <c r="E61" s="115" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="113" t="n"/>
-      <c r="C62" s="116" t="n"/>
-      <c r="E62" s="115" t="n"/>
+      <c r="A62" s="114" t="n"/>
+      <c r="C62" s="117" t="n"/>
+      <c r="E62" s="116" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="114" t="n"/>
-      <c r="C63" s="114" t="n"/>
-      <c r="E63" s="114" t="n"/>
+      <c r="A63" s="115" t="n"/>
+      <c r="C63" s="115" t="n"/>
+      <c r="E63" s="115" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="113" t="n"/>
-      <c r="C64" s="116" t="n"/>
-      <c r="E64" s="115" t="n"/>
+      <c r="A64" s="114" t="n"/>
+      <c r="C64" s="117" t="n"/>
+      <c r="E64" s="116" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="114" t="n"/>
-      <c r="C65" s="114" t="n"/>
-      <c r="E65" s="114" t="n"/>
+      <c r="A65" s="115" t="n"/>
+      <c r="C65" s="115" t="n"/>
+      <c r="E65" s="115" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="113" t="n"/>
-      <c r="C66" s="116" t="n"/>
-      <c r="E66" s="115" t="n"/>
+      <c r="A66" s="114" t="n"/>
+      <c r="C66" s="117" t="n"/>
+      <c r="E66" s="116" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="114" t="n"/>
-      <c r="C67" s="114" t="n"/>
-      <c r="E67" s="114" t="n"/>
+      <c r="A67" s="115" t="n"/>
+      <c r="C67" s="115" t="n"/>
+      <c r="E67" s="115" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="113" t="n"/>
-      <c r="C68" s="116" t="n"/>
-      <c r="E68" s="115" t="n"/>
+      <c r="A68" s="114" t="n"/>
+      <c r="C68" s="117" t="n"/>
+      <c r="E68" s="116" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="114" t="n"/>
-      <c r="C69" s="114" t="n"/>
-      <c r="E69" s="114" t="n"/>
+      <c r="A69" s="115" t="n"/>
+      <c r="C69" s="115" t="n"/>
+      <c r="E69" s="115" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="113" t="n"/>
-      <c r="C70" s="116" t="n"/>
-      <c r="E70" s="115" t="n"/>
+      <c r="A70" s="114" t="n"/>
+      <c r="C70" s="117" t="n"/>
+      <c r="E70" s="116" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="114" t="n"/>
-      <c r="C71" s="114" t="n"/>
-      <c r="E71" s="114" t="n"/>
+      <c r="A71" s="115" t="n"/>
+      <c r="C71" s="115" t="n"/>
+      <c r="E71" s="115" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="113" t="n"/>
-      <c r="C72" s="116" t="n"/>
-      <c r="E72" s="115" t="n"/>
+      <c r="A72" s="114" t="n"/>
+      <c r="C72" s="117" t="n"/>
+      <c r="E72" s="116" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="114" t="n"/>
-      <c r="C73" s="114" t="n"/>
-      <c r="E73" s="114" t="n"/>
+      <c r="A73" s="115" t="n"/>
+      <c r="C73" s="115" t="n"/>
+      <c r="E73" s="115" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="113" t="n"/>
-      <c r="C74" s="116" t="n"/>
-      <c r="E74" s="115" t="n"/>
+      <c r="A74" s="114" t="n"/>
+      <c r="C74" s="117" t="n"/>
+      <c r="E74" s="116" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="114" t="n"/>
-      <c r="C75" s="114" t="n"/>
-      <c r="E75" s="114" t="n"/>
+      <c r="A75" s="115" t="n"/>
+      <c r="C75" s="115" t="n"/>
+      <c r="E75" s="115" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="113" t="n"/>
-      <c r="C76" s="116" t="n"/>
-      <c r="E76" s="115" t="n"/>
+      <c r="A76" s="114" t="n"/>
+      <c r="C76" s="117" t="n"/>
+      <c r="E76" s="116" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="114" t="n"/>
-      <c r="C77" s="114" t="n"/>
-      <c r="E77" s="114" t="n"/>
+      <c r="A77" s="115" t="n"/>
+      <c r="C77" s="115" t="n"/>
+      <c r="E77" s="115" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="113" t="n"/>
-      <c r="C78" s="116" t="n"/>
-      <c r="E78" s="115" t="n"/>
+      <c r="A78" s="114" t="n"/>
+      <c r="C78" s="117" t="n"/>
+      <c r="E78" s="116" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="114" t="n"/>
-      <c r="C79" s="114" t="n"/>
-      <c r="E79" s="114" t="n"/>
+      <c r="A79" s="115" t="n"/>
+      <c r="C79" s="115" t="n"/>
+      <c r="E79" s="115" t="n"/>
     </row>
     <row r="82" ht="26" customHeight="1">
-      <c r="A82" s="67" t="inlineStr">
+      <c r="A82" s="68" t="inlineStr">
         <is>
           <t xml:space="preserve">  ПОСТОЯННЫЕ РАСХОДЫ (умная таблица tblПостоянные)</t>
         </is>
       </c>
     </row>
     <row r="83" ht="24" customHeight="1">
-      <c r="A83" s="117" t="inlineStr">
+      <c r="A83" s="118" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="B83" s="117" t="inlineStr">
+      <c r="B83" s="118" t="inlineStr">
         <is>
           <t>Зарплата</t>
         </is>
       </c>
-      <c r="C83" s="117" t="inlineStr">
+      <c r="C83" s="118" t="inlineStr">
         <is>
           <t>Аренда</t>
         </is>
       </c>
-      <c r="D83" s="117" t="inlineStr">
+      <c r="D83" s="118" t="inlineStr">
         <is>
           <t>Коммунальные</t>
         </is>
       </c>
-      <c r="E83" s="117" t="inlineStr">
+      <c r="E83" s="118" t="inlineStr">
         <is>
           <t>Налог</t>
         </is>
       </c>
-      <c r="F83" s="117" t="inlineStr">
+      <c r="F83" s="118" t="inlineStr">
         <is>
           <t>Маркетинг</t>
         </is>
       </c>
-      <c r="G83" s="117" t="inlineStr">
+      <c r="G83" s="118" t="inlineStr">
         <is>
           <t>Охрана</t>
         </is>
       </c>
-      <c r="H83" s="117" t="inlineStr">
+      <c r="H83" s="118" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
     </row>
     <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="118" t="inlineStr">
+      <c r="A84" s="119" t="inlineStr">
         <is>
           <t>Январь</t>
         </is>
       </c>
-      <c r="B84" s="119" t="n">
+      <c r="B84" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C84" s="119" t="n">
+      <c r="C84" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D84" s="119" t="n">
+      <c r="D84" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E84" s="119" t="n">
+      <c r="E84" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F84" s="119" t="n">
+      <c r="F84" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G84" s="119" t="n">
+      <c r="G84" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H84" s="120">
+      <c r="H84" s="121">
         <f>SUM(B84:G84)</f>
         <v/>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1">
-      <c r="A85" s="121" t="inlineStr">
+      <c r="A85" s="122" t="inlineStr">
         <is>
           <t>Февраль</t>
         </is>
       </c>
-      <c r="B85" s="119" t="n">
+      <c r="B85" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C85" s="119" t="n">
+      <c r="C85" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D85" s="119" t="n">
+      <c r="D85" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E85" s="119" t="n">
+      <c r="E85" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F85" s="119" t="n">
+      <c r="F85" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G85" s="119" t="n">
+      <c r="G85" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H85" s="120">
+      <c r="H85" s="121">
         <f>SUM(B85:G85)</f>
         <v/>
       </c>
     </row>
     <row r="86" ht="22" customHeight="1">
-      <c r="A86" s="118" t="inlineStr">
+      <c r="A86" s="119" t="inlineStr">
         <is>
           <t>Март</t>
         </is>
       </c>
-      <c r="B86" s="119" t="n">
+      <c r="B86" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C86" s="119" t="n">
+      <c r="C86" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D86" s="119" t="n">
+      <c r="D86" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E86" s="119" t="n">
+      <c r="E86" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F86" s="119" t="n">
+      <c r="F86" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G86" s="119" t="n">
+      <c r="G86" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H86" s="120">
+      <c r="H86" s="121">
         <f>SUM(B86:G86)</f>
         <v/>
       </c>
     </row>
     <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="121" t="inlineStr">
+      <c r="A87" s="122" t="inlineStr">
         <is>
           <t>Апрель</t>
         </is>
       </c>
-      <c r="B87" s="119" t="n">
+      <c r="B87" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C87" s="119" t="n">
+      <c r="C87" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D87" s="119" t="n">
+      <c r="D87" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E87" s="119" t="n">
+      <c r="E87" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F87" s="119" t="n">
+      <c r="F87" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G87" s="119" t="n">
+      <c r="G87" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H87" s="120">
+      <c r="H87" s="121">
         <f>SUM(B87:G87)</f>
         <v/>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="118" t="inlineStr">
+      <c r="A88" s="119" t="inlineStr">
         <is>
           <t>Май</t>
         </is>
       </c>
-      <c r="B88" s="119" t="n">
+      <c r="B88" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C88" s="119" t="n">
+      <c r="C88" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D88" s="119" t="n">
+      <c r="D88" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E88" s="119" t="n">
+      <c r="E88" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F88" s="119" t="n">
+      <c r="F88" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G88" s="119" t="n">
+      <c r="G88" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H88" s="120">
+      <c r="H88" s="121">
         <f>SUM(B88:G88)</f>
         <v/>
       </c>
     </row>
     <row r="89" ht="22" customHeight="1">
-      <c r="A89" s="121" t="inlineStr">
+      <c r="A89" s="122" t="inlineStr">
         <is>
           <t>Июнь</t>
         </is>
       </c>
-      <c r="B89" s="119" t="n">
+      <c r="B89" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C89" s="119" t="n">
+      <c r="C89" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D89" s="119" t="n">
+      <c r="D89" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E89" s="119" t="n">
+      <c r="E89" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F89" s="119" t="n">
+      <c r="F89" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G89" s="119" t="n">
+      <c r="G89" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H89" s="120">
+      <c r="H89" s="121">
         <f>SUM(B89:G89)</f>
         <v/>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="118" t="inlineStr">
+      <c r="A90" s="119" t="inlineStr">
         <is>
           <t>Июль</t>
         </is>
       </c>
-      <c r="B90" s="119" t="n">
+      <c r="B90" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C90" s="119" t="n">
+      <c r="C90" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D90" s="119" t="n">
+      <c r="D90" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E90" s="119" t="n">
+      <c r="E90" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F90" s="119" t="n">
+      <c r="F90" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G90" s="119" t="n">
+      <c r="G90" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H90" s="120">
+      <c r="H90" s="121">
         <f>SUM(B90:G90)</f>
         <v/>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1">
-      <c r="A91" s="121" t="inlineStr">
+      <c r="A91" s="122" t="inlineStr">
         <is>
           <t>Август</t>
         </is>
       </c>
-      <c r="B91" s="119" t="n">
+      <c r="B91" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C91" s="119" t="n">
+      <c r="C91" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D91" s="119" t="n">
+      <c r="D91" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E91" s="119" t="n">
+      <c r="E91" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F91" s="119" t="n">
+      <c r="F91" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G91" s="119" t="n">
+      <c r="G91" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H91" s="120">
+      <c r="H91" s="121">
         <f>SUM(B91:G91)</f>
         <v/>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1">
-      <c r="A92" s="118" t="inlineStr">
+      <c r="A92" s="119" t="inlineStr">
         <is>
           <t>Сентябрь</t>
         </is>
       </c>
-      <c r="B92" s="119" t="n">
+      <c r="B92" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C92" s="119" t="n">
+      <c r="C92" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D92" s="119" t="n">
+      <c r="D92" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E92" s="119" t="n">
+      <c r="E92" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F92" s="119" t="n">
+      <c r="F92" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G92" s="119" t="n">
+      <c r="G92" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H92" s="120">
+      <c r="H92" s="121">
         <f>SUM(B92:G92)</f>
         <v/>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="121" t="inlineStr">
+      <c r="A93" s="122" t="inlineStr">
         <is>
           <t>Октябрь</t>
         </is>
       </c>
-      <c r="B93" s="119" t="n">
+      <c r="B93" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C93" s="119" t="n">
+      <c r="C93" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D93" s="119" t="n">
+      <c r="D93" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E93" s="119" t="n">
+      <c r="E93" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F93" s="119" t="n">
+      <c r="F93" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G93" s="119" t="n">
+      <c r="G93" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H93" s="120">
+      <c r="H93" s="121">
         <f>SUM(B93:G93)</f>
         <v/>
       </c>
     </row>
     <row r="94" ht="22" customHeight="1">
-      <c r="A94" s="118" t="inlineStr">
+      <c r="A94" s="119" t="inlineStr">
         <is>
           <t>Ноябрь</t>
         </is>
       </c>
-      <c r="B94" s="119" t="n">
+      <c r="B94" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C94" s="119" t="n">
+      <c r="C94" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D94" s="119" t="n">
+      <c r="D94" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E94" s="119" t="n">
+      <c r="E94" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F94" s="119" t="n">
+      <c r="F94" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G94" s="119" t="n">
+      <c r="G94" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H94" s="120">
+      <c r="H94" s="121">
         <f>SUM(B94:G94)</f>
         <v/>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1">
-      <c r="A95" s="121" t="inlineStr">
+      <c r="A95" s="122" t="inlineStr">
         <is>
           <t>Декабрь</t>
         </is>
       </c>
-      <c r="B95" s="119" t="n">
+      <c r="B95" s="120" t="n">
         <v>540000</v>
       </c>
-      <c r="C95" s="119" t="n">
+      <c r="C95" s="120" t="n">
         <v>366000</v>
       </c>
-      <c r="D95" s="119" t="n">
+      <c r="D95" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="E95" s="119" t="n">
+      <c r="E95" s="120" t="n">
         <v>90000</v>
       </c>
-      <c r="F95" s="119" t="n">
+      <c r="F95" s="120" t="n">
         <v>30000</v>
       </c>
-      <c r="G95" s="119" t="n">
+      <c r="G95" s="120" t="n">
         <v>25000</v>
       </c>
-      <c r="H95" s="120">
+      <c r="H95" s="121">
         <f>SUM(B95:G95)</f>
         <v/>
       </c>
@@ -44985,7 +44986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46220,6 +46221,458 @@
       </c>
       <c r="D82" s="56">
         <f>B82-C82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="58" t="inlineStr">
+        <is>
+          <t>Общая выручка</t>
+        </is>
+      </c>
+      <c r="B100" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C100" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="58" t="inlineStr">
+        <is>
+          <t>Среднее в день</t>
+        </is>
+      </c>
+      <c r="B101" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)</f>
+        <v/>
+      </c>
+      <c r="C101" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="58" t="inlineStr">
+        <is>
+          <t>Среднее за смену</t>
+        </is>
+      </c>
+      <c r="B102" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)),0)</f>
+        <v/>
+      </c>
+      <c r="C102" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1)),0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="58" t="inlineStr">
+        <is>
+          <t>Лучший день</t>
+        </is>
+      </c>
+      <c r="B103" s="56">
+        <f>IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+        <v/>
+      </c>
+      <c r="C103" s="56">
+        <f>IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$C$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$D$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="58" t="inlineStr">
+        <is>
+          <t>Выплаты из кассы</t>
+        </is>
+      </c>
+      <c r="B104" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Выплата с кассы"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C104" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Выплата с кассы"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="58" t="inlineStr">
+        <is>
+          <t>Расхождений сумма</t>
+        </is>
+      </c>
+      <c r="B105" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C105" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="58" t="inlineStr">
+        <is>
+          <t>Кол-во расхождений</t>
+        </is>
+      </c>
+      <c r="B106">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)</f>
+        <v/>
+      </c>
+      <c r="C106">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Расхождение")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="58" t="inlineStr">
+        <is>
+          <t>Остаток кассы</t>
+        </is>
+      </c>
+      <c r="B107" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Касса")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C107" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Касса")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="58" t="inlineStr">
+        <is>
+          <t>Текущий долг</t>
+        </is>
+      </c>
+      <c r="B108" s="56">
+        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C108" s="56">
+        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="58" t="inlineStr">
+        <is>
+          <t>Взято в долг</t>
+        </is>
+      </c>
+      <c r="B109" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C109" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="58" t="inlineStr">
+        <is>
+          <t>Выплачено долгов</t>
+        </is>
+      </c>
+      <c r="B110" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Оплата долга"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C110" s="56">
+        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="58" t="inlineStr">
+        <is>
+          <t>К оплате (=долг)</t>
+        </is>
+      </c>
+      <c r="B111" s="56">
+        <f>IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+        <v/>
+      </c>
+      <c r="C111" s="56">
+        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="58" t="inlineStr">
+        <is>
+          <t>Закуп товара</t>
+        </is>
+      </c>
+      <c r="B112" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C112" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="58" t="inlineStr">
+        <is>
+          <t>Все расходы</t>
+        </is>
+      </c>
+      <c r="B113" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C113" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="58" t="inlineStr">
+        <is>
+          <t>Чистая прибыль</t>
+        </is>
+      </c>
+      <c r="B114" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+        <v/>
+      </c>
+      <c r="C114" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="58" t="inlineStr">
+        <is>
+          <t>Рентабельность %</t>
+        </is>
+      </c>
+      <c r="B115">
+        <f>IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+      <c r="C115">
+        <f>IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="58" t="inlineStr">
+        <is>
+          <t>Маржа %</t>
+        </is>
+      </c>
+      <c r="B116">
+        <f>IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+      <c r="C116">
+        <f>IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="58" t="inlineStr">
+        <is>
+          <t>Эффект. закупа (x)</t>
+        </is>
+      </c>
+      <c r="B117">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))),0)</f>
+        <v/>
+      </c>
+      <c r="C117">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="58" t="inlineStr">
+        <is>
+          <t>Нагрузка долга %</t>
+        </is>
+      </c>
+      <c r="B118">
+        <f>IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+      <c r="C118">
+        <f>IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="58" t="inlineStr">
+        <is>
+          <t>Ср. расход/день</t>
+        </is>
+      </c>
+      <c r="B119" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0))),0)</f>
+        <v/>
+      </c>
+      <c r="C119" s="56">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="58" t="inlineStr">
+        <is>
+          <t>Просроч. выплаты</t>
+        </is>
+      </c>
+      <c r="B120" s="56">
+        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)</f>
+        <v/>
+      </c>
+      <c r="C120" s="56">
+        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$C$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$D$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="58" t="inlineStr">
+        <is>
+          <t>Просроч. кол-во</t>
+        </is>
+      </c>
+      <c r="B121">
+        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*(КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003&lt;&gt;"")*(1)),0)</f>
+        <v/>
+      </c>
+      <c r="C121">
+        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$C$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$D$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*(КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003&lt;&gt;"")*(1)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="58" t="inlineStr">
+        <is>
+          <t>Выплачено %</t>
+        </is>
+      </c>
+      <c r="B122">
+        <f>IFERROR((IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$F$4:$F$1003),0))/MAX(1,(IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)))*100,0)</f>
+        <v/>
+      </c>
+      <c r="C122">
+        <f>50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="58" t="inlineStr">
+        <is>
+          <t>Закуп в долг %</t>
+        </is>
+      </c>
+      <c r="B123">
+        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Закуп товара")*(БАЗА_ДДС!$F$4:$F$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+        <v/>
+      </c>
+      <c r="C123">
+        <f>50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="58" t="inlineStr">
+        <is>
+          <t>Дней с данными</t>
+        </is>
+      </c>
+      <c r="B124">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="58" t="inlineStr">
+        <is>
+          <t>Всего операций</t>
+        </is>
+      </c>
+      <c r="B125">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="58" t="inlineStr">
+        <is>
+          <t>Макс. выручка/день</t>
+        </is>
+      </c>
+      <c r="B126" s="56">
+        <f>IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+        <v/>
+      </c>
+      <c r="C126" s="56">
+        <f>IFERROR(MINIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="58" t="inlineStr">
+        <is>
+          <t>Мин. выручка/день</t>
+        </is>
+      </c>
+      <c r="B127" s="56">
+        <f>IFERROR(MINIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="58" t="inlineStr">
+        <is>
+          <t>Иман (хозяин)</t>
+        </is>
+      </c>
+      <c r="B128" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Иман"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C128" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Иман"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="58" t="inlineStr">
+        <is>
+          <t>Списания+Возвраты</t>
+        </is>
+      </c>
+      <c r="B129" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Списание"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+      <c r="C129" s="56">
+        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Списание"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="58" t="inlineStr"/>
+      <c r="B130">
+        <f>0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="58" t="inlineStr"/>
+      <c r="B131">
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -46253,25 +46706,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>WAY MARKET — ДАШБОРД УПРАВЛЕНЧЕСКОГО УЧЁТА</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="59">
+      <c r="A2" s="60">
         <f>НАСТРОЙКИ!E5&amp;"  |  Данные с: "&amp;TEXT(НАСТРОЙКИ!E6,"DD.MM.YYYY")</f>
         <v/>
       </c>
-      <c r="F2" s="60">
+      <c r="F2" s="61">
         <f>"Всего записей: "&amp;COUNTA(БАЗА_ДДС!$A$4:$A$3003)&amp;"  |  Последнее обновление: "&amp;TEXT(NOW(),"DD.MM.YYYY HH:MM")</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr">
         <is>
           <t>ПЕРИОД:</t>
         </is>
@@ -46281,7 +46734,7 @@
           <t>Май</t>
         </is>
       </c>
-      <c r="D4" s="61" t="inlineStr">
+      <c r="D4" s="62" t="inlineStr">
         <is>
           <t>ГОД:</t>
         </is>
@@ -46289,11 +46742,11 @@
       <c r="E4" s="15" t="n">
         <v>2026</v>
       </c>
-      <c r="G4" s="62">
+      <c r="G4" s="63">
         <f>TEXT(A5,"DD.MM.YYYY")&amp;" — "&amp;TEXT(B5,"DD.MM.YYYY")</f>
         <v/>
       </c>
-      <c r="J4" s="63" t="inlineStr">
+      <c r="J4" s="64" t="inlineStr">
         <is>
           <t>[ОБНОВИТЬ] — кнопка VBA  |  Ctrl+Shift+D</t>
         </is>
@@ -46332,121 +46785,121 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="64" t="inlineStr">
+      <c r="A8" s="65" t="inlineStr">
         <is>
           <t>Общая выручка</t>
         </is>
       </c>
-      <c r="D8" s="64" t="inlineStr">
+      <c r="D8" s="65" t="inlineStr">
         <is>
           <t>Среднее в день</t>
         </is>
       </c>
-      <c r="G8" s="64" t="inlineStr">
+      <c r="G8" s="65" t="inlineStr">
         <is>
           <t>Среднее за смену</t>
         </is>
       </c>
-      <c r="J8" s="64" t="inlineStr">
+      <c r="J8" s="65" t="inlineStr">
         <is>
           <t>Лучший день</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="65">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="A9" s="66">
+        <f>ДАННЫЕ!$B$100</f>
         <v/>
       </c>
-      <c r="C9" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="C9" s="67">
+        <f>IF(ДАННЫЕ!$B$100&gt;ДАННЫЕ!$C$100,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D9" s="65">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)</f>
+      <c r="D9" s="66">
+        <f>ДАННЫЕ!$B$101</f>
         <v/>
       </c>
-      <c r="F9" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0))&gt;(IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)),"▲","▼")</f>
+      <c r="F9" s="67">
+        <f>IF(ДАННЫЕ!$B$101&gt;ДАННЫЕ!$C$101,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G9" s="65">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)),0)</f>
+      <c r="G9" s="66">
+        <f>ДАННЫЕ!$B$102</f>
         <v/>
       </c>
-      <c r="I9" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)),0))&gt;(IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1)),0)),0)),"▲","▼")</f>
+      <c r="I9" s="67">
+        <f>IF(ДАННЫЕ!$B$102&gt;ДАННЫЕ!$C$102,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J9" s="65">
-        <f>IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+      <c r="J9" s="66">
+        <f>ДАННЫЕ!$B$103</f>
         <v/>
       </c>
-      <c r="L9" s="66">
-        <f>IF((IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0))&gt;(IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$C$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$D$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)),"▲","▼")</f>
+      <c r="L9" s="67">
+        <f>IF(ДАННЫЕ!$B$103&gt;ДАННЫЕ!$C$103,"▲","▼")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="67" t="inlineStr">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t xml:space="preserve">  КОНТРОЛЬ КАССЫ</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="68" t="inlineStr">
+      <c r="A11" s="69" t="inlineStr">
         <is>
           <t>Выплаты из кассы</t>
         </is>
       </c>
-      <c r="D11" s="68" t="inlineStr">
+      <c r="D11" s="69" t="inlineStr">
         <is>
           <t>Расхождений сумма</t>
         </is>
       </c>
-      <c r="G11" s="68" t="inlineStr">
+      <c r="G11" s="69" t="inlineStr">
         <is>
           <t>Кол-во расхождений</t>
         </is>
       </c>
-      <c r="J11" s="68" t="inlineStr">
+      <c r="J11" s="69" t="inlineStr">
         <is>
           <t>Остаток кассы</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="69">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Выплата с кассы"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="A12" s="70">
+        <f>ДАННЫЕ!$B$104</f>
         <v/>
       </c>
-      <c r="C12" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Выплата с кассы"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Выплата с кассы"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="C12" s="67">
+        <f>IF(ДАННЫЕ!$B$104&gt;ДАННЫЕ!$C$104,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D12" s="69">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="D12" s="70">
+        <f>ДАННЫЕ!$B$105</f>
         <v/>
       </c>
-      <c r="F12" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="F12" s="67">
+        <f>IF(ДАННЫЕ!$B$105&gt;ДАННЫЕ!$C$105,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G12" s="70">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)</f>
+      <c r="G12" s="71">
+        <f>ДАННЫЕ!$B$106</f>
         <v/>
       </c>
-      <c r="I12" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расхождение"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Расхождение")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1)),0)),"▲","▼")</f>
+      <c r="I12" s="67">
+        <f>IF(ДАННЫЕ!$B$106&gt;ДАННЫЕ!$C$106,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J12" s="69">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Касса")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="J12" s="70">
+        <f>ДАННЫЕ!$B$107</f>
         <v/>
       </c>
-      <c r="L12" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Касса")*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Касса")*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="L12" s="67">
+        <f>IF(ДАННЫЕ!$B$107&gt;ДАННЫЕ!$C$107,"▲","▼")</f>
         <v/>
       </c>
     </row>
@@ -46458,58 +46911,58 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="71" t="inlineStr">
+      <c r="A14" s="72" t="inlineStr">
         <is>
           <t>Текущий долг</t>
         </is>
       </c>
-      <c r="D14" s="71" t="inlineStr">
+      <c r="D14" s="72" t="inlineStr">
         <is>
           <t>Взято в долг</t>
         </is>
       </c>
-      <c r="G14" s="71" t="inlineStr">
+      <c r="G14" s="72" t="inlineStr">
         <is>
           <t>Выплачено долгов</t>
         </is>
       </c>
-      <c r="J14" s="71" t="inlineStr">
+      <c r="J14" s="72" t="inlineStr">
         <is>
           <t>К оплате (=долг)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="72">
-        <f>IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="A15" s="73">
+        <f>ДАННЫЕ!$B$108</f>
         <v/>
       </c>
-      <c r="C15" s="66">
-        <f>IF((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="C15" s="67">
+        <f>IF(ДАННЫЕ!$B$108&gt;ДАННЫЕ!$C$108,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D15" s="72">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="D15" s="73">
+        <f>ДАННЫЕ!$B$109</f>
         <v/>
       </c>
-      <c r="F15" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Долг"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="F15" s="67">
+        <f>IF(ДАННЫЕ!$B$109&gt;ДАННЫЕ!$C$109,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G15" s="72">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Оплата долга"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="G15" s="73">
+        <f>ДАННЫЕ!$B$110</f>
         <v/>
       </c>
-      <c r="I15" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Оплата долга"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="I15" s="67">
+        <f>IF(ДАННЫЕ!$B$110&gt;ДАННЫЕ!$C$110,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J15" s="72">
-        <f>IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+      <c r="J15" s="73">
+        <f>ДАННЫЕ!$B$111</f>
         <v/>
       </c>
-      <c r="L15" s="66">
-        <f>IF((IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),0))&gt;(IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="L15" s="67">
+        <f>IF(ДАННЫЕ!$B$111&gt;ДАННЫЕ!$C$111,"▲","▼")</f>
         <v/>
       </c>
     </row>
@@ -46521,58 +46974,58 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="73" t="inlineStr">
+      <c r="A17" s="74" t="inlineStr">
         <is>
           <t>Закуп товара</t>
         </is>
       </c>
-      <c r="D17" s="73" t="inlineStr">
+      <c r="D17" s="74" t="inlineStr">
         <is>
           <t>Все расходы</t>
         </is>
       </c>
-      <c r="G17" s="73" t="inlineStr">
+      <c r="G17" s="74" t="inlineStr">
         <is>
           <t>Чистая прибыль</t>
         </is>
       </c>
-      <c r="J17" s="73" t="inlineStr">
+      <c r="J17" s="74" t="inlineStr">
         <is>
           <t>Рентабельность %</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="74">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="A18" s="75">
+        <f>ДАННЫЕ!$B$112</f>
         <v/>
       </c>
-      <c r="C18" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="C18" s="67">
+        <f>IF(ДАННЫЕ!$B$112&gt;ДАННЫЕ!$C$112,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D18" s="74">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="D18" s="75">
+        <f>ДАННЫЕ!$B$113</f>
         <v/>
       </c>
-      <c r="F18" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="F18" s="67">
+        <f>IF(ДАННЫЕ!$B$113&gt;ДАННЫЕ!$C$113,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G18" s="74">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0)</f>
+      <c r="G18" s="75">
+        <f>ДАННЫЕ!$B$114</f>
         <v/>
       </c>
-      <c r="I18" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))&gt;(IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0)),"▲","▼")</f>
+      <c r="I18" s="67">
+        <f>IF(ДАННЫЕ!$B$114&gt;ДАННЫЕ!$C$114,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J18" s="75">
-        <f>IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+      <c r="J18" s="76">
+        <f>ДАННЫЕ!$B$115</f>
         <v/>
       </c>
-      <c r="L18" s="66">
-        <f>IF((IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0))&gt;(IFERROR((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)),"▲","▼")</f>
+      <c r="L18" s="67">
+        <f>IF(ДАННЫЕ!$B$115&gt;ДАННЫЕ!$C$115,"▲","▼")</f>
         <v/>
       </c>
     </row>
@@ -46584,58 +47037,58 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="76" t="inlineStr">
+      <c r="A20" s="77" t="inlineStr">
         <is>
           <t>Маржа %</t>
         </is>
       </c>
-      <c r="D20" s="76" t="inlineStr">
+      <c r="D20" s="77" t="inlineStr">
         <is>
           <t>Эффект. закупа (x)</t>
         </is>
       </c>
-      <c r="G20" s="76" t="inlineStr">
+      <c r="G20" s="77" t="inlineStr">
         <is>
           <t>Нагрузка долга %</t>
         </is>
       </c>
-      <c r="J20" s="76" t="inlineStr">
+      <c r="J20" s="77" t="inlineStr">
         <is>
           <t>Ср. расход/день</t>
         </is>
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="77">
-        <f>IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+      <c r="A21" s="78">
+        <f>ДАННЫЕ!$B$116</f>
         <v/>
       </c>
-      <c r="C21" s="66">
-        <f>IF((IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0))&gt;(IFERROR(((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))-(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)),"▲","▼")</f>
+      <c r="C21" s="67">
+        <f>IF(ДАННЫЕ!$B$116&gt;ДАННЫЕ!$C$116,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D21" s="77">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))),0)</f>
+      <c r="D21" s="78">
+        <f>ДАННЫЕ!$B$117</f>
         <v/>
       </c>
-      <c r="F21" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))),0))&gt;(IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0))),0)),"▲","▼")</f>
+      <c r="F21" s="67">
+        <f>IF(ДАННЫЕ!$B$117&gt;ДАННЫЕ!$C$117,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G21" s="77">
-        <f>IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+      <c r="G21" s="78">
+        <f>ДАННЫЕ!$B$118</f>
         <v/>
       </c>
-      <c r="I21" s="66">
-        <f>IF((IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0))&gt;(IFERROR((IFERROR(НАСТРОЙКИ!E9+SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003)-SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Оплата долга")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)),"▲","▼")</f>
+      <c r="I21" s="67">
+        <f>IF(ДАННЫЕ!$B$118&gt;ДАННЫЕ!$C$118,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J21" s="78">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0))),0)</f>
+      <c r="J21" s="79">
+        <f>ДАННЫЕ!$B$119</f>
         <v/>
       </c>
-      <c r="L21" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0))),0))&gt;(IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)),0)),"▲","▼")</f>
+      <c r="L21" s="67">
+        <f>IF(ДАННЫЕ!$B$119&gt;ДАННЫЕ!$C$119,"▲","▼")</f>
         <v/>
       </c>
     </row>
@@ -46647,159 +47100,159 @@
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="79" t="inlineStr">
+      <c r="A23" s="80" t="inlineStr">
         <is>
           <t>Просроч. выплаты</t>
         </is>
       </c>
-      <c r="D23" s="79" t="inlineStr">
+      <c r="D23" s="80" t="inlineStr">
         <is>
           <t>Просроч. кол-во</t>
         </is>
       </c>
-      <c r="G23" s="79" t="inlineStr">
+      <c r="G23" s="80" t="inlineStr">
         <is>
           <t>Выплачено %</t>
         </is>
       </c>
-      <c r="J23" s="79" t="inlineStr">
+      <c r="J23" s="80" t="inlineStr">
         <is>
           <t>Закуп в долг %</t>
         </is>
       </c>
     </row>
     <row r="24" ht="38" customHeight="1">
-      <c r="A24" s="80">
-        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)</f>
+      <c r="A24" s="81">
+        <f>ДАННЫЕ!$B$120</f>
         <v/>
       </c>
-      <c r="C24" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0))&gt;(IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$C$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$D$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)),"▲","▼")</f>
+      <c r="C24" s="67">
+        <f>IF(ДАННЫЕ!$B$120&gt;ДАННЫЕ!$C$120,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D24" s="81">
-        <f>IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*(КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003&lt;&gt;"")*(1)),0)</f>
+      <c r="D24" s="82">
+        <f>ДАННЫЕ!$B$121</f>
         <v/>
       </c>
-      <c r="F24" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*(КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003&lt;&gt;"")*(1)),0))&gt;(IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$C$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$D$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$G$4:$G$1003="Просрочено")*(КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003&lt;&gt;"")*(1)),0)),"▲","▼")</f>
+      <c r="F24" s="67">
+        <f>IF(ДАННЫЕ!$B$121&gt;ДАННЫЕ!$C$121,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G24" s="81">
-        <f>IFERROR((IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$F$4:$F$1003),0))/MAX(1,(IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)))*100,0)</f>
+      <c r="G24" s="82">
+        <f>ДАННЫЕ!$B$122</f>
         <v/>
       </c>
-      <c r="I24" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$F$4:$F$1003),0))/MAX(1,(IFERROR(SUMPRODUCT((КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&gt;=$A$5)*(КАЛЕНДАРЬ_ВЫПЛАТ!$A$4:$A$1003&lt;=$B$5)*КАЛЕНДАРЬ_ВЫПЛАТ!$D$4:$D$1003),0)))*100,0))&gt;(50),"▲","▼")</f>
+      <c r="I24" s="67">
+        <f>IF(ДАННЫЕ!$B$122&gt;ДАННЫЕ!$C$122,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J24" s="81">
-        <f>IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Закуп товара")*(БАЗА_ДДС!$F$4:$F$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0)</f>
+      <c r="J24" s="82">
+        <f>ДАННЫЕ!$B$123</f>
         <v/>
       </c>
-      <c r="L24" s="66">
-        <f>IF((IFERROR((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Закуп товара")*(БАЗА_ДДС!$F$4:$F$3003="Долг")*БАЗА_ДДС!$G$4:$G$3003),0))/MAX(1,(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*((БАЗА_ДДС!$E$4:$E$3003="Закуп товара"))*БАЗА_ДДС!$G$4:$G$3003),0)))*100,0))&gt;(50),"▲","▼")</f>
+      <c r="L24" s="67">
+        <f>IF(ДАННЫЕ!$B$123&gt;ДАННЫЕ!$C$123,"▲","▼")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="82" t="inlineStr">
+      <c r="A25" s="83" t="inlineStr">
         <is>
           <t xml:space="preserve">  СТАТИСТИКА ПЕРИОДА</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="83" t="inlineStr">
+      <c r="A26" s="84" t="inlineStr">
         <is>
           <t>Дней с данными</t>
         </is>
       </c>
-      <c r="D26" s="83" t="inlineStr">
+      <c r="D26" s="84" t="inlineStr">
         <is>
           <t>Всего операций</t>
         </is>
       </c>
-      <c r="G26" s="83" t="inlineStr">
+      <c r="G26" s="84" t="inlineStr">
         <is>
           <t>Макс. выручка/день</t>
         </is>
       </c>
-      <c r="J26" s="83" t="inlineStr">
+      <c r="J26" s="84" t="inlineStr">
         <is>
           <t>Мин. выручка/день</t>
         </is>
       </c>
     </row>
     <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="84">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$D$4:$D$3003="Доход")*(БАЗА_ДДС!$G$4:$G$3003&lt;&gt;"")*(1/COUNTIFS(БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$A$4:$A$3003,БАЗА_ДДС!$D$4:$D$3003,"Доход"))),0)</f>
+      <c r="A27" s="85">
+        <f>ДАННЫЕ!$B$124</f>
         <v/>
       </c>
-      <c r="C27" s="85" t="inlineStr"/>
-      <c r="D27" s="84">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Доход"))*((БАЗА_ДДС!$G$4:$G$3003&lt;&gt;""))*(1)),0)</f>
+      <c r="C27" s="86" t="inlineStr"/>
+      <c r="D27" s="85">
+        <f>ДАННЫЕ!$B$125</f>
         <v/>
       </c>
-      <c r="F27" s="85" t="inlineStr"/>
-      <c r="G27" s="86">
-        <f>IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+      <c r="F27" s="86" t="inlineStr"/>
+      <c r="G27" s="87">
+        <f>ДАННЫЕ!$B$126</f>
         <v/>
       </c>
-      <c r="I27" s="66">
-        <f>IF((IFERROR(MAXIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0))&gt;(IFERROR(MINIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)),"▲","▼")</f>
+      <c r="I27" s="67">
+        <f>IF(ДАННЫЕ!$B$126&gt;ДАННЫЕ!$C$126,"▲","▼")</f>
         <v/>
       </c>
-      <c r="J27" s="86">
-        <f>IFERROR(MINIFS(БАЗА_ДДС!$G$4:$G$3003,БАЗА_ДДС!$A$4:$A$3003,"&gt;="&amp;$A$5,БАЗА_ДДС!$A$4:$A$3003,"&lt;="&amp;$B$5,БАЗА_ДДС!$D$4:$D$3003,"Доход"),0)</f>
+      <c r="J27" s="87">
+        <f>ДАННЫЕ!$B$127</f>
         <v/>
       </c>
-      <c r="L27" s="85" t="inlineStr"/>
+      <c r="L27" s="86" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="83" t="inlineStr">
+      <c r="A28" s="84" t="inlineStr">
         <is>
           <t>Иман (хозяин)</t>
         </is>
       </c>
-      <c r="D28" s="83" t="inlineStr">
+      <c r="D28" s="84" t="inlineStr">
         <is>
           <t>Списания+Возвраты</t>
         </is>
       </c>
-      <c r="G28" s="83" t="inlineStr"/>
-      <c r="J28" s="83" t="inlineStr"/>
+      <c r="G28" s="84" t="inlineStr"/>
+      <c r="J28" s="84" t="inlineStr"/>
     </row>
     <row r="29" ht="38" customHeight="1">
-      <c r="A29" s="86">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Иман"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="A29" s="87">
+        <f>ДАННЫЕ!$B$128</f>
         <v/>
       </c>
-      <c r="C29" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Иман"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Иман"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="C29" s="67">
+        <f>IF(ДАННЫЕ!$B$128&gt;ДАННЫЕ!$C$128,"▲","▼")</f>
         <v/>
       </c>
-      <c r="D29" s="86">
-        <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Списание"))*БАЗА_ДДС!$G$4:$G$3003),0)</f>
+      <c r="D29" s="87">
+        <f>ДАННЫЕ!$B$129</f>
         <v/>
       </c>
-      <c r="F29" s="66">
-        <f>IF((IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Списание"))*БАЗА_ДДС!$G$4:$G$3003),0))&gt;(IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$C$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$D$5))*((БАЗА_ДДС!$D$4:$D$3003="Списание"))*БАЗА_ДДС!$G$4:$G$3003),0)),"▲","▼")</f>
+      <c r="F29" s="67">
+        <f>IF(ДАННЫЕ!$B$129&gt;ДАННЫЕ!$C$129,"▲","▼")</f>
         <v/>
       </c>
-      <c r="G29" s="84">
-        <f>0</f>
+      <c r="G29" s="85">
+        <f>ДАННЫЕ!$B$130</f>
         <v/>
       </c>
-      <c r="I29" s="85" t="inlineStr"/>
-      <c r="J29" s="84">
-        <f>0</f>
+      <c r="I29" s="86" t="inlineStr"/>
+      <c r="J29" s="85">
+        <f>ДАННЫЕ!$B$131</f>
         <v/>
       </c>
-      <c r="L29" s="85" t="inlineStr"/>
+      <c r="L29" s="86" t="inlineStr"/>
     </row>
     <row r="30" ht="10" customHeight="1">
-      <c r="A30" s="87" t="n"/>
+      <c r="A30" s="88" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -46809,62 +47262,62 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="88" t="inlineStr">
+      <c r="A32" s="89" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B32" s="88" t="inlineStr">
+      <c r="B32" s="89" t="inlineStr">
         <is>
           <t>Сумма</t>
         </is>
       </c>
-      <c r="C32" s="88" t="inlineStr">
+      <c r="C32" s="89" t="inlineStr">
         <is>
           <t>Доля %</t>
         </is>
       </c>
-      <c r="D32" s="88" t="inlineStr">
+      <c r="D32" s="89" t="inlineStr">
         <is>
           <t>Гистограмма</t>
         </is>
       </c>
-      <c r="E32" s="88" t="inlineStr">
+      <c r="E32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F32" s="88" t="inlineStr">
+      <c r="F32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="88" t="inlineStr">
+      <c r="G32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H32" s="88" t="inlineStr">
+      <c r="H32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I32" s="88" t="inlineStr">
+      <c r="I32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J32" s="88" t="inlineStr">
+      <c r="J32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K32" s="88" t="inlineStr">
+      <c r="K32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L32" s="88" t="inlineStr">
+      <c r="L32" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -46876,15 +47329,15 @@
           <t>Закуп товара</t>
         </is>
       </c>
-      <c r="B33" s="89">
+      <c r="B33" s="90">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Закуп товара")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C33" s="90">
+      <c r="C33" s="91">
         <f>IFERROR(B33/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D33" s="91">
+      <c r="D33" s="92">
         <f>IFERROR(REPT("|",MAX(1,INT(B33/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46895,15 +47348,15 @@
           <t>Зарплата</t>
         </is>
       </c>
-      <c r="B34" s="92">
+      <c r="B34" s="93">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Зарплата")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C34" s="93">
+      <c r="C34" s="94">
         <f>IFERROR(B34/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D34" s="94">
+      <c r="D34" s="95">
         <f>IFERROR(REPT("|",MAX(1,INT(B34/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46914,15 +47367,15 @@
           <t>Аренда</t>
         </is>
       </c>
-      <c r="B35" s="95">
+      <c r="B35" s="96">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Аренда")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C35" s="90">
+      <c r="C35" s="91">
         <f>IFERROR(B35/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D35" s="91">
+      <c r="D35" s="92">
         <f>IFERROR(REPT("|",MAX(1,INT(B35/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46933,15 +47386,15 @@
           <t>Коммунальные</t>
         </is>
       </c>
-      <c r="B36" s="92">
+      <c r="B36" s="93">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Коммунальные")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C36" s="93">
+      <c r="C36" s="94">
         <f>IFERROR(B36/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D36" s="94">
+      <c r="D36" s="95">
         <f>IFERROR(REPT("|",MAX(1,INT(B36/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46952,15 +47405,15 @@
           <t>Налог</t>
         </is>
       </c>
-      <c r="B37" s="95">
+      <c r="B37" s="96">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Налог")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C37" s="90">
+      <c r="C37" s="91">
         <f>IFERROR(B37/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D37" s="91">
+      <c r="D37" s="92">
         <f>IFERROR(REPT("|",MAX(1,INT(B37/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46971,15 +47424,15 @@
           <t>ГСМ</t>
         </is>
       </c>
-      <c r="B38" s="92">
+      <c r="B38" s="93">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="ГСМ")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C38" s="93">
+      <c r="C38" s="94">
         <f>IFERROR(B38/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D38" s="94">
+      <c r="D38" s="95">
         <f>IFERROR(REPT("|",MAX(1,INT(B38/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -46990,15 +47443,15 @@
           <t>Расходный материал</t>
         </is>
       </c>
-      <c r="B39" s="95">
+      <c r="B39" s="96">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Расходный материал")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C39" s="90">
+      <c r="C39" s="91">
         <f>IFERROR(B39/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D39" s="91">
+      <c r="D39" s="92">
         <f>IFERROR(REPT("|",MAX(1,INT(B39/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -47009,15 +47462,15 @@
           <t>Маркетинг</t>
         </is>
       </c>
-      <c r="B40" s="92">
+      <c r="B40" s="93">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Маркетинг")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C40" s="93">
+      <c r="C40" s="94">
         <f>IFERROR(B40/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D40" s="94">
+      <c r="D40" s="95">
         <f>IFERROR(REPT("|",MAX(1,INT(B40/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -47028,15 +47481,15 @@
           <t>Охрана</t>
         </is>
       </c>
-      <c r="B41" s="95">
+      <c r="B41" s="96">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Охрана")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C41" s="90">
+      <c r="C41" s="91">
         <f>IFERROR(B41/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D41" s="91">
+      <c r="D41" s="92">
         <f>IFERROR(REPT("|",MAX(1,INT(B41/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
@@ -47047,21 +47500,21 @@
           <t>Прочие расходы</t>
         </is>
       </c>
-      <c r="B42" s="92">
+      <c r="B42" s="93">
         <f>IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5)*(БАЗА_ДДС!$E$4:$E$3003="Прочие расходы")*БАЗА_ДДС!$G$4:$G$3003),0)</f>
         <v/>
       </c>
-      <c r="C42" s="93">
+      <c r="C42" s="94">
         <f>IFERROR(B42/IFERROR(SUMPRODUCT((БАЗА_ДДС!$A$4:$A$3003&gt;=$A$5)*(БАЗА_ДДС!$A$4:$A$3003&lt;=$B$5))*((БАЗА_ДДС!$D$4:$D$3003="Расход"))*БАЗА_ДДС!$G$4:$G$3003),0)*100,0)</f>
         <v/>
       </c>
-      <c r="D42" s="94">
+      <c r="D42" s="95">
         <f>IFERROR(REPT("|",MAX(1,INT(B42/MAX($B$33:$B$42)*20))),"")</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="8" customHeight="1">
-      <c r="A43" s="87" t="n"/>
+      <c r="A43" s="88" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Fix НАСТРОЙКИ tblФиксРасходы: col A rows 13-16 now editable (locked=False + INP fill)
Category name cells (Аренда/Налоги/Интернет/Охрана) were missing prot(False)
and had gray fill instead of blue input fill — looked and behaved like locked labels.
</commit_message>
<xml_diff>
--- a/WAY_MARKET_v9.xlsx
+++ b/WAY_MARKET_v9.xlsx
@@ -3086,7 +3086,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Аренда</t>
         </is>
@@ -3096,7 +3096,7 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Налоги</t>
         </is>
@@ -3106,7 +3106,7 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Интернет</t>
         </is>
@@ -3116,7 +3116,7 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Охрана</t>
         </is>

</xml_diff>